<commit_message>
Add VincoliTemporali: finestre orarie per-operatore via Excel
Nuovo foglio opzionale VincoliTemporali (Nome, Data inizio, Data fine,
Ora inizio, Ora fine, Note). Nell'intervallo indicato l'operatore puo'
lavorare solo turni interamente contenuti nella finestra oraria.

- TimeConstraint dataclass + parsing in load_input (retro-compat: foglio
  assente -> constraints vuoti)
- apply_time_constraints filtra le shift options nei 3 call site di
  build_schedule (Zetema combo, Non-Zetema greedy, rebalance)
- _forced_rest_by_constraints: giorni con finestra incompatibile sono
  marcati come riposo forzato in generate_rest_days (log [INFO])
- Vincoli multipli sovrapposti -> intersezione delle finestre
- Template aggiornato con 2 righe esempio e note
- 9 test in test_vincoli_temporali.py (parsing, default, intersezione,
  rest forzato, operatore sconosciuto, date/ore invalide)

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/input_turni_template.xlsx
+++ b/input_turni_template.xlsx
@@ -11,6 +11,7 @@
     <sheet name="Periodo" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="Copertura" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="Assenze" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="VincoliTemporali" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1073,11 +1074,12 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B5"/>
+  <dimension ref="A1:C5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
     <col width="20" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
@@ -1091,6 +1093,11 @@
           <t>Data assenza</t>
         </is>
       </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Tipo assenza</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -1101,6 +1108,11 @@
       <c r="B2" s="4" t="n">
         <v>45756</v>
       </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>Ferie</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -1111,11 +1123,147 @@
       <c r="B3" s="4" t="n">
         <v>45761</v>
       </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>Malattia</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
         <is>
-          <t>⚠ Inserire una riga per ogni giorno di assenza.  Il nome deve corrispondere esattamente al foglio Personale.</t>
+          <t>⚠ Inserire una riga per ogni giorno di assenza.  Il nome deve corrispondere esattamente al foglio Personale.  Tipo: es. Ferie, Malattia, Permesso (opzionale, default: Assenza).</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F7"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="25" customWidth="1" min="1" max="1"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="30" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="30" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Nome operatore</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Data inizio</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Data fine</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Ora inizio</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Ora fine</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Note</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Mario Rossi</t>
+        </is>
+      </c>
+      <c r="B2" s="4" t="n">
+        <v>45778</v>
+      </c>
+      <c r="C2" s="4" t="n">
+        <v>45808</v>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>07:00</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>14:00</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>Solo mattina</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>Anna Bianchi</t>
+        </is>
+      </c>
+      <c r="B3" s="4" t="n">
+        <v>45818</v>
+      </c>
+      <c r="C3" s="4" t="n">
+        <v>45818</v>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>13:00</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>20:00</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>Visita medica mattina</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t>⚠ Foglio OPZIONALE. Nell'intervallo [Data inizio, Data fine] l'operatore può lavorare SOLO turni interamente contenuti in [Ora inizio, Ora fine].</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="3" t="inlineStr">
+        <is>
+          <t>Data fine vuota → singolo giorno. Ore vuote → nessun vincolo orario (solo nota). Più righe stesso operatore → intersezione delle finestre nei giorni sovrapposti.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="3" t="inlineStr">
+        <is>
+          <t>Eliminare righe di esempio se non servono. Se tutto il foglio è vuoto, nessun vincolo è applicato.</t>
         </is>
       </c>
     </row>

</xml_diff>